<commit_message>
Classify Sunpro structural supplies under lumber
</commit_message>
<xml_diff>
--- a/Deploy/site_ove/sub-docs/sunpro/files/3f7fdd322032-Sunpro_Bid_vs_Invoices.xlsx
+++ b/Deploy/site_ove/sub-docs/sunpro/files/3f7fdd322032-Sunpro_Bid_vs_Invoices.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sunpro" sheetId="1" r:id="Re3d75fb0c7264c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sunpro" sheetId="1" r:id="R3334d093bbd948fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -551,16 +551,49 @@
       <x:c r="G3" t="n">
         <x:v>4531.05</x:v>
       </x:c>
+      <x:c r="I3" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="J3" t="n">
+        <x:v>27.74</x:v>
+      </x:c>
+      <x:c r="K3" t="n">
+        <x:v>-2162.05</x:v>
+      </x:c>
+      <x:c r="L3" t="n">
+        <x:v>2162.05</x:v>
+      </x:c>
+      <x:c r="M3" t="n">
+        <x:v>2162.05</x:v>
+      </x:c>
+      <x:c r="N3" t="n">
+        <x:v>4030.29</x:v>
+      </x:c>
+      <x:c r="O3" t="n">
+        <x:v>1962.25</x:v>
+      </x:c>
+      <x:c r="P3" t="n">
+        <x:v>131.4</x:v>
+      </x:c>
+      <x:c r="Q3" t="n">
+        <x:v>128.61</x:v>
+      </x:c>
+      <x:c r="S3" t="n">
+        <x:v>-3447.8</x:v>
+      </x:c>
       <x:c r="T3" s="2" t="n">
-        <x:v>4531.05</x:v>
+        <x:f>SUM(G3:S3)+W3</x:f>
+        <x:v>10157.5</x:v>
       </x:c>
       <x:c r="U3" s="2" t="n">
-        <x:v>70468.95</x:v>
-      </x:c>
-      <x:c r="V3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Inv 3890718 (6/29/26): framing lumber pkg — studs, plates, T&amp;G OSB, LSL band board, Simpson pins, delivery+fuel. $4,251.31 + $279.74 tax = $4,531.05. Job 746 Liberty Lane, SO 19267935. Due 7/30/26.</x:t>
-        </x:is>
+        <x:f>F3-T3</x:f>
+        <x:v>64842.5</x:v>
+      </x:c>
+      <x:c r="V3" t="str">
+        <x:v>Inv 3890718 (6/29/26): framing lumber pkg — studs, plates, T&amp;G OSB, LSL band board, Simpson pins, delivery+fuel. $4,251.31 + $279.74 tax = $4,531.05. Job 746 Liberty Lane, SO 19267935. Due 7/30/26. Inv 3894241 (7/1/26): Simpson SDS wood screws box, $87.12 + $5.88 tax = $93.00. Job 746 Liberty Lane. Due 8/1/26. Credit 255676 (7/30/26): price-correction credit against invoice 3920799 / order 19430770, rebar, strap tie holdowns, anchor bolts, and bearing plates, total credit $2,162.05. Inv 3920799 (7/30/26): same materials delivered to 746 Liberty Lane, $2,025.34 + $136.71 tax = $2,162.05, due 8/30/26. Inv 3921247 (7/31/26): corrected payable hardware and rebar invoice after the 7/30 invoice/credit pair; rebar, strap tie holdowns, anchor bolts, and bearing plates for 746 Liberty Lane. $2,025.34 + $136.71 tax = $2,162.05, due 8/31/26. Inv 3897876 (7/6/26): Simpson strong-wall anchor bolt/templates plus delivery/fuel for 746 Liberty Lane, $3,783.55 + $246.74 tax = $4,030.29, due 8/6/26. Inv 3899137 (7/7/26): Sunpro material/delivery charge for 746 Liberty Lane, $1,844.23 + $118.02 tax = $1,962.25, due 8/7/26. Inv 3899710 (7/8/26): Sunpro material charge for 746 Liberty Lane, $123.09 + $8.31 tax = $131.40, due 8/8/26. Inv 3902213 (7/10/26): Sunpro material charge for 746 Liberty Lane, $120.48 + $8.13 tax = $128.61, due 8/10/26. Credit 257064 (8/20/26): return/credit against invoice 3897876 / order 19312055, Simpson Strong Wall shearwall materials for 746 Liberty Lane. Total credit $3,447.80 ($3,229.79 materials + $218.01 tax). Invoice 3984650: $538.91, hardware, dated October 8, 2026; due November 8. No payment recorded. Craig classified these structural materials as Lumber on October 20, 2026.</x:v>
+      </x:c>
+      <x:c r="W3" t="n">
+        <x:v>538.91</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -668,10 +701,8 @@
       <x:c r="A7" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hardware</x:t>
-        </x:is>
+      <x:c r="B7" t="str">
+        <x:v>Door &amp; Bath Hardware</x:v>
       </x:c>
       <x:c r="C7" t="n">
         <x:v>1</x:v>
@@ -687,50 +718,28 @@
       <x:c r="F7" t="n">
         <x:v>5500</x:v>
       </x:c>
-      <x:c r="I7" t="n">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="J7" s="2" t="n">
-        <x:v>27.74</x:v>
-      </x:c>
-      <x:c r="K7" s="2" t="n">
-        <x:v>-2162.05</x:v>
-      </x:c>
-      <x:c r="L7" s="2" t="n">
-        <x:v>2162.05</x:v>
-      </x:c>
-      <x:c r="M7" s="2" t="n">
-        <x:v>2162.05</x:v>
-      </x:c>
-      <x:c r="N7" s="2" t="n">
-        <x:v>4030.29</x:v>
-      </x:c>
-      <x:c r="O7" s="2" t="n">
-        <x:v>1962.25</x:v>
-      </x:c>
-      <x:c r="P7" s="2" t="n">
-        <x:v>131.4</x:v>
-      </x:c>
-      <x:c r="Q7" s="2" t="n">
-        <x:v>128.61</x:v>
-      </x:c>
-      <x:c r="S7" t="n">
-        <x:v>-3447.8</x:v>
-      </x:c>
+      <x:c r="I7"/>
+      <x:c r="J7" s="2"/>
+      <x:c r="K7" s="2"/>
+      <x:c r="L7" s="2"/>
+      <x:c r="M7" s="2"/>
+      <x:c r="N7" s="2"/>
+      <x:c r="O7" s="2"/>
+      <x:c r="P7" s="2"/>
+      <x:c r="Q7" s="2"/>
+      <x:c r="S7"/>
       <x:c r="T7" s="2" t="n">
         <x:f>SUM(G7:S7)+W7</x:f>
-        <x:v>5626.45</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="U7" s="2" t="n">
         <x:f>F7-T7</x:f>
-        <x:v>-126.44999999999982</x:v>
+        <x:v>5500</x:v>
       </x:c>
       <x:c r="V7" t="str">
-        <x:v>Inv 3894241 (7/1/26): Simpson SDS wood screws box, $87.12 + $5.88 tax = $93.00. Job 746 Liberty Lane. Due 8/1/26. Credit 255676 (7/30/26): price-correction credit against invoice 3920799 / order 19430770, rebar, strap tie holdowns, anchor bolts, and bearing plates, total credit $2,162.05. Inv 3920799 (7/30/26): same materials delivered to 746 Liberty Lane, $2,025.34 + $136.71 tax = $2,162.05, due 8/30/26. Inv 3921247 (7/31/26): corrected payable hardware and rebar invoice after the 7/30 invoice/credit pair; rebar, strap tie holdowns, anchor bolts, and bearing plates for 746 Liberty Lane. $2,025.34 + $136.71 tax = $2,162.05, due 8/31/26. Inv 3897876 (7/6/26): Simpson strong-wall anchor bolt/templates plus delivery/fuel for 746 Liberty Lane, $3,783.55 + $246.74 tax = $4,030.29, due 8/6/26. Inv 3899137 (7/7/26): Sunpro material/delivery charge for 746 Liberty Lane, $1,844.23 + $118.02 tax = $1,962.25, due 8/7/26. Inv 3899710 (7/8/26): Sunpro material charge for 746 Liberty Lane, $123.09 + $8.31 tax = $131.40, due 8/8/26. Inv 3902213 (7/10/26): Sunpro material charge for 746 Liberty Lane, $120.48 + $8.13 tax = $128.61, due 8/10/26. Credit 257064 (8/20/26): return/credit against invoice 3897876 / order 19312055, Simpson Strong Wall shearwall materials for 746 Liberty Lane. Total credit $3,447.80 ($3,229.79 materials + $218.01 tax). Invoice 3984650: $538.91, hardware, dated October 8, 2026; due November 8. No payment recorded.</x:v>
-      </x:c>
-      <x:c r="W7" t="n">
-        <x:v>538.91</x:v>
-      </x:c>
+        <x:v>No door or bath hardware purchased. Structural supplies reclassified to Lumber.</x:v>
+      </x:c>
+      <x:c r="W7"/>
     </x:row>
     <x:row r="9">
       <x:c r="B9" t="inlineStr">

</xml_diff>